<commit_message>
Add harvRipe into obs func Gna25
</commit_message>
<xml_diff>
--- a/Tests/Validation/Wheat/UoM_WheatProject/Gnarwarre2025_Observed.xlsx
+++ b/Tests/Validation/Wheat/UoM_WheatProject/Gnarwarre2025_Observed.xlsx
@@ -1525,6 +1525,11 @@
       <c r="P57">
         <v>867.3578156468332</v>
       </c>
+      <c r="AN57" t="inlineStr">
+        <is>
+          <t>HarvestRipe</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2883,6 +2888,11 @@
       <c r="P133">
         <v>626.7094634131316</v>
       </c>
+      <c r="AN133" t="inlineStr">
+        <is>
+          <t>HarvestRipe</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4241,6 +4251,11 @@
       <c r="P209">
         <v>775.0568630311111</v>
       </c>
+      <c r="AN209" t="inlineStr">
+        <is>
+          <t>HarvestRipe</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -5579,6 +5594,11 @@
       <c r="P283">
         <v>618.8171024987198</v>
       </c>
+      <c r="AN283" t="inlineStr">
+        <is>
+          <t>HarvestRipe</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
@@ -6914,6 +6934,11 @@
       <c r="P357">
         <v>716.5621476701518</v>
       </c>
+      <c r="AN357" t="inlineStr">
+        <is>
+          <t>HarvestRipe</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
@@ -8238,6 +8263,11 @@
       </c>
       <c r="P430">
         <v>659.9216611697351</v>
+      </c>
+      <c r="AN430" t="inlineStr">
+        <is>
+          <t>HarvestRipe</t>
+        </is>
       </c>
     </row>
     <row r="431">

</xml_diff>